<commit_message>
Benchmark snapshot: Survey Processing workbooks corrected for M-O1-LT agreement
Both copies refreshed from the IP folder (22 September 2026): the 60
formulas in 9 Type C Scoring C6:G17 now take MAXIFS over each decision
type's own import rows, replacing the N() wrapper Excel evaluated as the
first row alone. Formula-cell count unchanged at 4,562; the listing carries
the new template hash. Recorded in the IP folder's DECISIONS.md item 8.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/benchmarks/Survey Processing and Scoring Workbook.xlsx
+++ b/docs/benchmarks/Survey Processing and Scoring Workbook.xlsx
@@ -51397,23 +51397,23 @@
         <v/>
       </c>
       <c r="C6" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$32)*N('4 Import Leadership'!$I$5:$I$154)))/$B6,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$32)/$B6,""))</f>
         <v/>
       </c>
       <c r="D6" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$32)*N('4 Import Leadership'!$J$5:$J$154)))/$B6,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$32)/$B6,""))</f>
         <v/>
       </c>
       <c r="E6" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$32)*N('4 Import Leadership'!$K$5:$K$154)))/$B6,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$32)/$B6,""))</f>
         <v/>
       </c>
       <c r="F6" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$32)*N('4 Import Leadership'!$L$5:$L$154)))/$B6,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$32)/$B6,""))</f>
         <v/>
       </c>
       <c r="G6" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$32)*N('4 Import Leadership'!$M$5:$M$154)))/$B6,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$32="",$B6=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$32)/$B6,""))</f>
         <v/>
       </c>
       <c r="H6" s="19" t="str">
@@ -51431,23 +51431,23 @@
         <v/>
       </c>
       <c r="C7" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$33)*N('4 Import Leadership'!$I$5:$I$154)))/$B7,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$33)/$B7,""))</f>
         <v/>
       </c>
       <c r="D7" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$33)*N('4 Import Leadership'!$J$5:$J$154)))/$B7,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$33)/$B7,""))</f>
         <v/>
       </c>
       <c r="E7" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$33)*N('4 Import Leadership'!$K$5:$K$154)))/$B7,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$33)/$B7,""))</f>
         <v/>
       </c>
       <c r="F7" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$33)*N('4 Import Leadership'!$L$5:$L$154)))/$B7,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$33)/$B7,""))</f>
         <v/>
       </c>
       <c r="G7" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$33)*N('4 Import Leadership'!$M$5:$M$154)))/$B7,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$33="",$B7=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$33)/$B7,""))</f>
         <v/>
       </c>
       <c r="H7" s="19" t="str">
@@ -51465,23 +51465,23 @@
         <v/>
       </c>
       <c r="C8" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$34)*N('4 Import Leadership'!$I$5:$I$154)))/$B8,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$34)/$B8,""))</f>
         <v/>
       </c>
       <c r="D8" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$34)*N('4 Import Leadership'!$J$5:$J$154)))/$B8,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$34)/$B8,""))</f>
         <v/>
       </c>
       <c r="E8" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$34)*N('4 Import Leadership'!$K$5:$K$154)))/$B8,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$34)/$B8,""))</f>
         <v/>
       </c>
       <c r="F8" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$34)*N('4 Import Leadership'!$L$5:$L$154)))/$B8,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$34)/$B8,""))</f>
         <v/>
       </c>
       <c r="G8" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$34)*N('4 Import Leadership'!$M$5:$M$154)))/$B8,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$34="",$B8=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$34)/$B8,""))</f>
         <v/>
       </c>
       <c r="H8" s="19" t="str">
@@ -51499,23 +51499,23 @@
         <v/>
       </c>
       <c r="C9" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$35)*N('4 Import Leadership'!$I$5:$I$154)))/$B9,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$35)/$B9,""))</f>
         <v/>
       </c>
       <c r="D9" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$35)*N('4 Import Leadership'!$J$5:$J$154)))/$B9,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$35)/$B9,""))</f>
         <v/>
       </c>
       <c r="E9" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$35)*N('4 Import Leadership'!$K$5:$K$154)))/$B9,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$35)/$B9,""))</f>
         <v/>
       </c>
       <c r="F9" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$35)*N('4 Import Leadership'!$L$5:$L$154)))/$B9,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$35)/$B9,""))</f>
         <v/>
       </c>
       <c r="G9" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$35)*N('4 Import Leadership'!$M$5:$M$154)))/$B9,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$35="",$B9=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$35)/$B9,""))</f>
         <v/>
       </c>
       <c r="H9" s="19" t="str">
@@ -51533,23 +51533,23 @@
         <v/>
       </c>
       <c r="C10" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$36)*N('4 Import Leadership'!$I$5:$I$154)))/$B10,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$36)/$B10,""))</f>
         <v/>
       </c>
       <c r="D10" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$36)*N('4 Import Leadership'!$J$5:$J$154)))/$B10,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$36)/$B10,""))</f>
         <v/>
       </c>
       <c r="E10" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$36)*N('4 Import Leadership'!$K$5:$K$154)))/$B10,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$36)/$B10,""))</f>
         <v/>
       </c>
       <c r="F10" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$36)*N('4 Import Leadership'!$L$5:$L$154)))/$B10,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$36)/$B10,""))</f>
         <v/>
       </c>
       <c r="G10" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$36)*N('4 Import Leadership'!$M$5:$M$154)))/$B10,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$36="",$B10=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$36)/$B10,""))</f>
         <v/>
       </c>
       <c r="H10" s="19" t="str">
@@ -51567,23 +51567,23 @@
         <v/>
       </c>
       <c r="C11" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$37)*N('4 Import Leadership'!$I$5:$I$154)))/$B11,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$37)/$B11,""))</f>
         <v/>
       </c>
       <c r="D11" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$37)*N('4 Import Leadership'!$J$5:$J$154)))/$B11,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$37)/$B11,""))</f>
         <v/>
       </c>
       <c r="E11" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$37)*N('4 Import Leadership'!$K$5:$K$154)))/$B11,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$37)/$B11,""))</f>
         <v/>
       </c>
       <c r="F11" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$37)*N('4 Import Leadership'!$L$5:$L$154)))/$B11,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$37)/$B11,""))</f>
         <v/>
       </c>
       <c r="G11" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$37)*N('4 Import Leadership'!$M$5:$M$154)))/$B11,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$37="",$B11=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$37)/$B11,""))</f>
         <v/>
       </c>
       <c r="H11" s="19" t="str">
@@ -51601,23 +51601,23 @@
         <v/>
       </c>
       <c r="C12" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$38)*N('4 Import Leadership'!$I$5:$I$154)))/$B12,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$38)/$B12,""))</f>
         <v/>
       </c>
       <c r="D12" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$38)*N('4 Import Leadership'!$J$5:$J$154)))/$B12,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$38)/$B12,""))</f>
         <v/>
       </c>
       <c r="E12" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$38)*N('4 Import Leadership'!$K$5:$K$154)))/$B12,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$38)/$B12,""))</f>
         <v/>
       </c>
       <c r="F12" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$38)*N('4 Import Leadership'!$L$5:$L$154)))/$B12,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$38)/$B12,""))</f>
         <v/>
       </c>
       <c r="G12" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$38)*N('4 Import Leadership'!$M$5:$M$154)))/$B12,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$38="",$B12=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$38)/$B12,""))</f>
         <v/>
       </c>
       <c r="H12" s="19" t="str">
@@ -51635,23 +51635,23 @@
         <v/>
       </c>
       <c r="C13" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$39)*N('4 Import Leadership'!$I$5:$I$154)))/$B13,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$39)/$B13,""))</f>
         <v/>
       </c>
       <c r="D13" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$39)*N('4 Import Leadership'!$J$5:$J$154)))/$B13,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$39)/$B13,""))</f>
         <v/>
       </c>
       <c r="E13" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$39)*N('4 Import Leadership'!$K$5:$K$154)))/$B13,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$39)/$B13,""))</f>
         <v/>
       </c>
       <c r="F13" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$39)*N('4 Import Leadership'!$L$5:$L$154)))/$B13,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$39)/$B13,""))</f>
         <v/>
       </c>
       <c r="G13" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$39)*N('4 Import Leadership'!$M$5:$M$154)))/$B13,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$39="",$B13=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$39)/$B13,""))</f>
         <v/>
       </c>
       <c r="H13" s="19" t="str">
@@ -51669,23 +51669,23 @@
         <v/>
       </c>
       <c r="C14" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$40)*N('4 Import Leadership'!$I$5:$I$154)))/$B14,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$40)/$B14,""))</f>
         <v/>
       </c>
       <c r="D14" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$40)*N('4 Import Leadership'!$J$5:$J$154)))/$B14,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$40)/$B14,""))</f>
         <v/>
       </c>
       <c r="E14" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$40)*N('4 Import Leadership'!$K$5:$K$154)))/$B14,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$40)/$B14,""))</f>
         <v/>
       </c>
       <c r="F14" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$40)*N('4 Import Leadership'!$L$5:$L$154)))/$B14,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$40)/$B14,""))</f>
         <v/>
       </c>
       <c r="G14" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$40)*N('4 Import Leadership'!$M$5:$M$154)))/$B14,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$40="",$B14=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$40)/$B14,""))</f>
         <v/>
       </c>
       <c r="H14" s="19" t="str">
@@ -51703,23 +51703,23 @@
         <v/>
       </c>
       <c r="C15" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$41)*N('4 Import Leadership'!$I$5:$I$154)))/$B15,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$41)/$B15,""))</f>
         <v/>
       </c>
       <c r="D15" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$41)*N('4 Import Leadership'!$J$5:$J$154)))/$B15,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$41)/$B15,""))</f>
         <v/>
       </c>
       <c r="E15" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$41)*N('4 Import Leadership'!$K$5:$K$154)))/$B15,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$41)/$B15,""))</f>
         <v/>
       </c>
       <c r="F15" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$41)*N('4 Import Leadership'!$L$5:$L$154)))/$B15,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$41)/$B15,""))</f>
         <v/>
       </c>
       <c r="G15" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$41)*N('4 Import Leadership'!$M$5:$M$154)))/$B15,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$41="",$B15=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$41)/$B15,""))</f>
         <v/>
       </c>
       <c r="H15" s="19" t="str">
@@ -51737,23 +51737,23 @@
         <v/>
       </c>
       <c r="C16" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$42)*N('4 Import Leadership'!$I$5:$I$154)))/$B16,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$42)/$B16,""))</f>
         <v/>
       </c>
       <c r="D16" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$42)*N('4 Import Leadership'!$J$5:$J$154)))/$B16,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$42)/$B16,""))</f>
         <v/>
       </c>
       <c r="E16" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$42)*N('4 Import Leadership'!$K$5:$K$154)))/$B16,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$42)/$B16,""))</f>
         <v/>
       </c>
       <c r="F16" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$42)*N('4 Import Leadership'!$L$5:$L$154)))/$B16,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$42)/$B16,""))</f>
         <v/>
       </c>
       <c r="G16" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$42)*N('4 Import Leadership'!$M$5:$M$154)))/$B16,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$42="",$B16=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$42)/$B16,""))</f>
         <v/>
       </c>
       <c r="H16" s="19" t="str">
@@ -51771,23 +51771,23 @@
         <v/>
       </c>
       <c r="C17" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$43)*N('4 Import Leadership'!$I$5:$I$154)))/$B17,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$I$5:$I$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$43)/$B17,""))</f>
         <v/>
       </c>
       <c r="D17" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$43)*N('4 Import Leadership'!$J$5:$J$154)))/$B17,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$J$5:$J$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$43)/$B17,""))</f>
         <v/>
       </c>
       <c r="E17" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$43)*N('4 Import Leadership'!$K$5:$K$154)))/$B17,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$K$5:$K$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$43)/$B17,""))</f>
         <v/>
       </c>
       <c r="F17" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$43)*N('4 Import Leadership'!$L$5:$L$154)))/$B17,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$L$5:$L$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$43)/$B17,""))</f>
         <v/>
       </c>
       <c r="G17" s="19" t="str">
-        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(SUMPRODUCT(MAX(('4 Import Leadership'!$B$5:$B$154='1 Setup &amp; Keys'!$D$43)*N('4 Import Leadership'!$M$5:$M$154)))/$B17,""))</f>
+        <f aca="false">IF(OR('1 Setup &amp; Keys'!$D$43="",$B17=0),"",IFERROR(_xlfn.MAXIFS('4 Import Leadership'!$M$5:$M$154,'4 Import Leadership'!$B$5:$B$154,'1 Setup &amp; Keys'!$D$43)/$B17,""))</f>
         <v/>
       </c>
       <c r="H17" s="19" t="str">

</xml_diff>